<commit_message>
updated reason xlsx file
Signed-off-by: Abhi <abhishek.shankarcs@gmail.com>
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/reason_list.xlsx
+++ b/mosip_master/xlsx/reason_list.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="105">
   <si>
     <t xml:space="preserve">lang_code</t>
   </si>
@@ -56,6 +56,15 @@
   </si>
   <si>
     <t xml:space="preserve">TRUE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VPM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avge-Photo Mismatch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mismatch between the Avge and Photo</t>
   </si>
   <si>
     <t xml:space="preserve">GPM</t>
@@ -462,7 +471,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F1048576"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr defaultColWidth="8.4296875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="48.84"/>
@@ -581,7 +590,7 @@
         <v>22</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>10</v>
@@ -595,16 +604,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>11</v>
@@ -624,7 +633,7 @@
         <v>27</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>11</v>
@@ -635,16 +644,16 @@
         <v>6</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>11</v>
@@ -655,16 +664,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>11</v>
@@ -672,19 +681,19 @@
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>34</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>11</v>
@@ -692,16 +701,16 @@
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>10</v>
@@ -712,16 +721,16 @@
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>10</v>
@@ -732,16 +741,16 @@
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>18</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>10</v>
@@ -752,16 +761,16 @@
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>10</v>
@@ -772,19 +781,19 @@
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>11</v>
@@ -792,19 +801,19 @@
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>11</v>
@@ -812,19 +821,19 @@
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>11</v>
@@ -832,39 +841,39 @@
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D20" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>48</v>
       </c>
+      <c r="D20" s="4" t="s">
+        <v>48</v>
+      </c>
       <c r="E20" s="4" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>11</v>
@@ -872,16 +881,16 @@
     </row>
     <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E21" s="4" t="s">
         <v>10</v>
@@ -892,16 +901,16 @@
     </row>
     <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>10</v>
@@ -912,16 +921,16 @@
     </row>
     <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>18</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>10</v>
@@ -932,16 +941,16 @@
     </row>
     <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>10</v>
@@ -952,19 +961,19 @@
     </row>
     <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>11</v>
@@ -972,19 +981,19 @@
     </row>
     <row r="26" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>11</v>
@@ -992,19 +1001,19 @@
     </row>
     <row r="27" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>11</v>
@@ -1012,39 +1021,39 @@
     </row>
     <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D29" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C29" s="5" t="s">
         <v>62</v>
       </c>
+      <c r="D29" s="5" t="s">
+        <v>62</v>
+      </c>
       <c r="E29" s="4" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>11</v>
@@ -1052,16 +1061,16 @@
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E30" s="4" t="s">
         <v>10</v>
@@ -1072,16 +1081,16 @@
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E31" s="4" t="s">
         <v>10</v>
@@ -1092,16 +1101,16 @@
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>18</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>10</v>
@@ -1110,18 +1119,18 @@
         <v>11</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C33" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>69</v>
+      <c r="C33" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>71</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>10</v>
@@ -1132,19 +1141,19 @@
     </row>
     <row r="34" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>70</v>
+        <v>24</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>72</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>11</v>
@@ -1152,19 +1161,19 @@
     </row>
     <row r="35" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>11</v>
@@ -1172,19 +1181,19 @@
     </row>
     <row r="36" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>11</v>
@@ -1192,39 +1201,39 @@
     </row>
     <row r="37" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>73</v>
+        <v>31</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>75</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="D38" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C38" s="6" t="s">
         <v>76</v>
       </c>
+      <c r="D38" s="6" t="s">
+        <v>76</v>
+      </c>
       <c r="E38" s="4" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="F38" s="1" t="s">
         <v>11</v>
@@ -1232,16 +1241,16 @@
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E39" s="4" t="s">
         <v>10</v>
@@ -1252,16 +1261,16 @@
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E40" s="4" t="s">
         <v>10</v>
@@ -1272,16 +1281,16 @@
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>18</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E41" s="4" t="s">
         <v>10</v>
@@ -1290,18 +1299,18 @@
         <v>11</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="D42" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>85</v>
       </c>
       <c r="E42" s="4" t="s">
         <v>10</v>
@@ -1312,19 +1321,19 @@
     </row>
     <row r="43" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F43" s="1" t="s">
         <v>11</v>
@@ -1332,19 +1341,19 @@
     </row>
     <row r="44" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>11</v>
@@ -1352,19 +1361,19 @@
     </row>
     <row r="45" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F45" s="1" t="s">
         <v>11</v>
@@ -1372,39 +1381,39 @@
     </row>
     <row r="46" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F46" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="D47" s="4" t="s">
         <v>90</v>
       </c>
+      <c r="D47" s="6" t="s">
+        <v>90</v>
+      </c>
       <c r="E47" s="4" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="F47" s="1" t="s">
         <v>11</v>
@@ -1412,16 +1421,16 @@
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E48" s="4" t="s">
         <v>10</v>
@@ -1432,16 +1441,16 @@
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E49" s="4" t="s">
         <v>10</v>
@@ -1452,16 +1461,16 @@
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>18</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E50" s="4" t="s">
         <v>10</v>
@@ -1472,16 +1481,16 @@
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B51" s="4" t="s">
         <v>21</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E51" s="4" t="s">
         <v>10</v>
@@ -1490,41 +1499,41 @@
         <v>11</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C52" s="6" t="s">
-        <v>98</v>
+        <v>24</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>100</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F52" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B53" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C53" s="4" t="s">
-        <v>99</v>
+      <c r="C53" s="6" t="s">
+        <v>101</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F53" s="1" t="s">
         <v>11</v>
@@ -1532,19 +1541,19 @@
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F54" s="1" t="s">
         <v>11</v>
@@ -1552,29 +1561,48 @@
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F55" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>